<commit_message>
chore: stage all remaining changes before rebase and push to GitHub
</commit_message>
<xml_diff>
--- a/BASES DATOS/usuarios_aphis-usda_new_web_app_updated.xlsx
+++ b/BASES DATOS/usuarios_aphis-usda_new_web_app_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\tb-yucatan_new_web_app\BASES DATOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFBD24EB-5C0E-4BFD-BD36-ABAB2BA1BE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4C5D9C-FB48-48E0-ABB0-F60F958C52B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="51">
   <si>
     <t>nombre</t>
   </si>
@@ -85,18 +85,9 @@
     <t>MunozSader#99</t>
   </si>
   <si>
-    <t xml:space="preserve">Gerardo Solís Pasos </t>
-  </si>
-  <si>
-    <t>gerardo.solis@yucatan.gob.mx</t>
-  </si>
-  <si>
     <t>Estatal</t>
   </si>
   <si>
-    <t>SederYucSOLIS@2024</t>
-  </si>
-  <si>
     <t>Juan Carlos Rodríguez Andrade</t>
   </si>
   <si>
@@ -182,24 +173,6 @@
   </si>
   <si>
     <t>Siniiga2025!</t>
-  </si>
-  <si>
-    <t>Oscar Correa</t>
-  </si>
-  <si>
-    <t>oscar.correa@cefppy.org</t>
-  </si>
-  <si>
-    <t>CorreaCefppy#7</t>
-  </si>
-  <si>
-    <t>Ivonne Galera Chan</t>
-  </si>
-  <si>
-    <t>ivonne.galera@vas.org</t>
-  </si>
-  <si>
-    <t>VasGalera$123</t>
   </si>
 </sst>
 </file>
@@ -576,15 +549,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.19921875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.59765625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -604,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -621,7 +594,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -638,7 +611,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -655,7 +628,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -672,15 +645,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
         <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
@@ -689,7 +662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -697,7 +670,7 @@
         <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
         <v>27</v>
@@ -706,7 +679,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -714,7 +687,7 @@
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D8" t="s">
         <v>30</v>
@@ -723,7 +696,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -731,7 +704,7 @@
         <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="D9" t="s">
         <v>33</v>
@@ -740,7 +713,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -748,24 +721,24 @@
         <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
         <v>36</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
       </c>
       <c r="D11" t="s">
         <v>40</v>
@@ -774,7 +747,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -782,7 +755,7 @@
         <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
         <v>43</v>
@@ -791,7 +764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -799,7 +772,7 @@
         <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D13" t="s">
         <v>46</v>
@@ -808,7 +781,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -816,70 +789,19 @@
         <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" t="s">
-        <v>52</v>
-      </c>
-      <c r="D15" t="s">
-        <v>53</v>
-      </c>
-      <c r="E15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" t="s">
-        <v>39</v>
-      </c>
-      <c r="D17" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F17" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F5 A6:F7 A9:F14 A8:B8 D8:F8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>